<commit_message>
ajout des graphiques dans les doc word
</commit_message>
<xml_diff>
--- a/Input/redaction_template.xlsx
+++ b/Input/redaction_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="179">
   <si>
     <t>condition</t>
   </si>
@@ -480,26 +480,6 @@
     <t>p13_neutre</t>
   </si>
   <si>
-    <t xml:space="preserve">قراءة: في {lib_mois_courant } {annee_courante } انخفض الرقم الاستدلالي للأثمان عند الاستهلاك
-ب {evol_non_alim_12mois} % مقارنة بشهر {lib_mois_courant } {annee_m12 } </t>
-  </si>
-  <si>
-    <t>Lecture: En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation a décru de {evol_non_alim_12mois}% par rapport à {lib_mois_courant} {annee_m12}</t>
-  </si>
-  <si>
-    <t>Reading: In {lib_mois_courant} {annee_courante}, the consumer price index decreased by {evol_non_alim_12mois}% compared to {lib_mois_courant} {annee_m12}</t>
-  </si>
-  <si>
-    <t>Lecture: En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation a augmenté de {evol_non_alim_12mois}% par rapport à {lib_mois_courant} {annee_m12}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">قراءة: في {lib_mois_courant } {annee_courante } ارتفع الرقم الاستدلالي للأثمان عند الاستهلاك
-ب {evol_non_alim_12mois} % مقارنة بشهر {lib_mois_courant } {annee_m12 } </t>
-  </si>
-  <si>
-    <t>Reading: In {lib_mois_courant} {annee_courante}, the consumer price index increased by {evol_non_alim_12mois}% compared to {lib_mois_courant} {annee_m12}</t>
-  </si>
-  <si>
     <t>Reading: In {lib_mois_courant} {annee_courante}, the consumer price index decreased stagnated compared to {lib_mois_courant} {annee_m12}</t>
   </si>
   <si>
@@ -523,6 +503,86 @@
   </si>
   <si>
     <t xml:space="preserve"> Évolution de la variation mensuelle (%) de l’indice des prix à la consommation</t>
+  </si>
+  <si>
+    <t>p16</t>
+  </si>
+  <si>
+    <t>p16_neutre</t>
+  </si>
+  <si>
+    <t>p16_moins</t>
+  </si>
+  <si>
+    <t>p16_plus</t>
+  </si>
+  <si>
+    <t>Lecture: En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation a augmenté de {evol_1mois}% par rapport à {lib_mois_m1} {annee_m1}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">قراءة: في {lib_mois_courant } {annee_courante } ارتفع الرقم الاستدلالي للأثمان عند الاستهلاك
+ب {evol_1mois} % مقارنة بشهر {lib_mois_m1} {annee_m1 } </t>
+  </si>
+  <si>
+    <t>Reading: In {lib_mois_courant} {annee_courante}, the consumer price index increased by {evol_1mois}% compared to {lib_mois_m1} {annee_m1}</t>
+  </si>
+  <si>
+    <t>Lecture: En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation a diminué de {evol_1mois}% par rapport à {lib_mois_m1} {annee_m1}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">قراءة: في {lib_mois_courant } {annee_courante } انخفظ الرقم الاستدلالي للأثمان عند الاستهلاك
+ب {evol_1mois} % مقارنة بشهر {lib_mois_m1} {annee_m1 } </t>
+  </si>
+  <si>
+    <t>Reading: In {lib_mois_courant} {annee_courante}, the consumer price index decreased by {evol_1mois}% compared to {lib_mois_m1} {annee_m1}</t>
+  </si>
+  <si>
+    <t>evol_1mois &lt; 0</t>
+  </si>
+  <si>
+    <t>evol_1mois &gt; 0</t>
+  </si>
+  <si>
+    <t>evol_1mois = 0</t>
+  </si>
+  <si>
+    <t>Lecture: En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation a gardé la même valeur par rapport à {lib_mois_m1} {annee_m1}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">قراءة: في {lib_mois_courant } {annee_courante } حافظ الرقم الاستدلالي للأثمان عند الاستهلاك
+على نفس القيمة مقارنة بشهر {lib_mois_m1 } {annee_m1 } </t>
+  </si>
+  <si>
+    <t>Reading: In {lib_mois_courant} {annee_courante}, the consumer price index decreased stagnated compared to {lib_mois_m1} {annee_m1}</t>
+  </si>
+  <si>
+    <t>evol_12mois &gt; 0</t>
+  </si>
+  <si>
+    <t>evol_12mois &lt; 0</t>
+  </si>
+  <si>
+    <t>evol_12mois = 0</t>
+  </si>
+  <si>
+    <t>Lecture: En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation a augmenté de {evol_12mois}% par rapport à {lib_mois_courant} {annee_m12}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">قراءة: في {lib_mois_courant } {annee_courante } ارتفع الرقم الاستدلالي للأثمان عند الاستهلاك
+ب {evol_12mois} % مقارنة بشهر {lib_mois_courant } {annee_m12 } </t>
+  </si>
+  <si>
+    <t>Reading: In {lib_mois_courant} {annee_courante}, the consumer price index increased by {evol_12mois}% compared to {lib_mois_courant} {annee_m12}</t>
+  </si>
+  <si>
+    <t>Reading: In {lib_mois_courant} {annee_courante}, the consumer price index decreased by {evol_12mois}% compared to {lib_mois_courant} {annee_m12}</t>
+  </si>
+  <si>
+    <t>Lecture: En {lib_mois_courant} {annee_courante}, l'indice des prix à la consommation a décru de {evol_12mois}% par rapport à {lib_mois_courant} {annee_m12}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">قراءة: في {lib_mois_courant } {annee_courante } انخفض الرقم الاستدلالي للأثمان عند الاستهلاك
+{evol_12mois} % مقارنة بشهر {lib_mois_courant } {annee_m12 } </t>
   </si>
 </sst>
 </file>
@@ -868,7 +928,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.85546875" style="1"/>
@@ -1447,16 +1507,16 @@
         <v>141</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="60">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="45">
       <c r="A31" s="1" t="s">
         <v>142</v>
       </c>
@@ -1464,19 +1524,19 @@
         <v>143</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>127</v>
+        <v>170</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>149</v>
+        <v>173</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>150</v>
+        <v>174</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="60">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="45">
       <c r="A32" s="1" t="s">
         <v>142</v>
       </c>
@@ -1484,16 +1544,16 @@
         <v>144</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>147</v>
+        <v>177</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>146</v>
+        <v>178</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>148</v>
+        <v>176</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="45">
@@ -1504,33 +1564,93 @@
         <v>145</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>125</v>
+        <v>172</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="30">
       <c r="A34" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="45">
+      <c r="A35" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="45">
+      <c r="A36" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="45">
+      <c r="A37" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>158</v>
+      <c r="C37" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
correction probleme rapport par ville
</commit_message>
<xml_diff>
--- a/Input/redaction_template.xlsx
+++ b/Input/redaction_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="187">
   <si>
     <t>condition</t>
   </si>
@@ -584,12 +584,56 @@
     <t xml:space="preserve">قراءة: في {lib_mois_courant } {annee_courante } انخفض الرقم الاستدلالي للأثمان عند الاستهلاك
 {evol_12mois} % مقارنة بشهر {lib_mois_courant } {annee_m12 } </t>
   </si>
+  <si>
+    <t>p17</t>
+  </si>
+  <si>
+    <t>Indice des prix à la consommation de la {ville}: {lib_mois_courant}  {annee_courante} (base 2017: 100)</t>
+  </si>
+  <si>
+    <t>Consumer price index for the {ville}: {lib_mois_courant}  {annee_courante} (2017 base: 100)</t>
+  </si>
+  <si>
+    <t>الرقم الاستدلالي للأثمان عند الاستهلاك {ville} {lib_mois_courant } :{annee_courante } (أساس 2017:100)</t>
+  </si>
+  <si>
+    <t>p20</t>
+  </si>
+  <si>
+    <t>Source: High Commission for Planning, Department of Statistics - National consumer price survey</t>
+  </si>
+  <si>
+    <t>Source: Haut-Commissariat au Plan, Direction de la Statistique – Enquête Nationale sur les Prix à la Consommation.</t>
+  </si>
+  <si>
+    <r>
+      <t>المصدر</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="TimesNewRomanPS-BoldMT"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color rgb="FF8D4355"/>
+        <rFont val="TimesNewRomanPS-BoldMT"/>
+      </rPr>
+      <t>المندوبية السامية للتخطيط، مديرية الإحصاء -البحث الوطني حول الأثمان عند الاستهلاك</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -614,6 +658,18 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="TimesNewRomanPSMT"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF8D4355"/>
+      <name val="TimesNewRomanPS-BoldMT"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="TimesNewRomanPS-BoldMT"/>
     </font>
   </fonts>
   <fills count="2">
@@ -928,7 +984,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8.85546875" style="1"/>
@@ -1651,6 +1707,40 @@
       </c>
       <c r="F37" s="1" t="s">
         <v>169</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="30">
+      <c r="A38" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="45">
+      <c r="A39" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>